<commit_message>
[feat] add Gauss Seidel
</commit_message>
<xml_diff>
--- a/Excel Autorizado - Cálculo Numérico.xlsx
+++ b/Excel Autorizado - Cálculo Numérico.xlsx
@@ -1,22 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gusta\Documents\codes\excel-calc-num-baixar\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2DD18506-B13C-4264-A9BF-468D4772133E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{2F65629C-D8E6-4631-B153-A7A717F4EA21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" firstSheet="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sistemas Lineares" sheetId="1" r:id="rId1"/>
-    <sheet name="Bissecção" sheetId="2" r:id="rId2"/>
-    <sheet name="Lagrange" sheetId="3" r:id="rId3"/>
-    <sheet name="Newton" sheetId="4" r:id="rId4"/>
+    <sheet name="Sistemas Lineares - Jacobi" sheetId="1" r:id="rId1"/>
+    <sheet name="Sistemas Lineares - Seidel" sheetId="6" r:id="rId2"/>
+    <sheet name="Bissecção" sheetId="2" r:id="rId3"/>
+    <sheet name="Lagrange" sheetId="3" r:id="rId4"/>
+    <sheet name="Newton" sheetId="4" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -42,10 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="45">
-  <si>
-    <t>SISTEMAS LINEARES</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="47">
   <si>
     <t>Interação</t>
   </si>
@@ -177,6 +175,15 @@
   </si>
   <si>
     <t>Ordem 4</t>
+  </si>
+  <si>
+    <t>SISTEMAS LINEARES - JACOBI</t>
+  </si>
+  <si>
+    <t>SISTEMAS LINEARES - SEIDEL</t>
+  </si>
+  <si>
+    <t>Δx3</t>
   </si>
 </sst>
 </file>
@@ -450,7 +457,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -614,11 +621,196 @@
     <xf numFmtId="0" fontId="2" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="64">
+  <dxfs count="79">
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF000000"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+        <right/>
+        <top/>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+        <right/>
+        <top/>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+        <right/>
+        <top/>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border>
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border>
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border>
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF000000"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+        <right/>
+        <top/>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+        <right/>
+        <top/>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+        <right/>
+        <top/>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border>
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF000000"/>
+        </right>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF000000"/>
@@ -652,6 +844,29 @@
         <color rgb="FF000000"/>
       </font>
       <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="center" wrapText="0"/>
+      <border>
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF000000"/>
+        </right>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" wrapText="0"/>
+      <border>
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF000000"/>
+        </right>
+      </border>
     </dxf>
     <dxf>
       <font>
@@ -805,7 +1020,9 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <alignment horizontal="center" wrapText="0"/>
       <border>
         <left style="thin">
@@ -820,6 +1037,9 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <alignment horizontal="center" wrapText="0"/>
       <border>
         <left style="thin">
@@ -831,10 +1051,31 @@
       </border>
     </dxf>
     <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <alignment horizontal="center" wrapText="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color theme="0"/>
+      </font>
+      <alignment horizontal="center" wrapText="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border>
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border>
         <left style="thin">
           <color rgb="FF000000"/>
@@ -846,117 +1087,6 @@
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" wrapText="0"/>
-      <border>
-        <left style="thin">
-          <color rgb="FF000000"/>
-        </left>
-        <right style="thin">
-          <color rgb="FF000000"/>
-        </right>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" wrapText="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color theme="0"/>
-      </font>
-      <alignment horizontal="center" wrapText="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border>
-        <left style="thin">
-          <color rgb="FF000000"/>
-        </left>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border>
-        <left style="thin">
-          <color rgb="FF000000"/>
-        </left>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border>
-        <left style="thin">
-          <color rgb="FF000000"/>
-        </left>
-        <right style="thin">
-          <color rgb="FF000000"/>
-        </right>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border>
-        <left style="thin">
-          <color rgb="FF000000"/>
-        </left>
-        <right style="thin">
-          <color rgb="FF000000"/>
-        </right>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border>
-        <left style="thin">
-          <color rgb="FF000000"/>
-        </left>
-        <right style="thin">
-          <color rgb="FF000000"/>
-        </right>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border>
-        <left style="thin">
-          <color rgb="FF000000"/>
-        </left>
-        <right style="thin">
-          <color rgb="FF000000"/>
-        </right>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border>
-        <left style="thin">
-          <color rgb="FF000000"/>
-        </left>
-        <right style="thin">
-          <color rgb="FF000000"/>
-        </right>
-      </border>
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1072,18 +1202,18 @@
   <tableStyles count="3" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9">
     <tableStyle name="Table Style 1" pivot="0" count="0" xr9:uid="{38A84C71-7F09-4571-8F02-A4CE054D42F6}"/>
     <tableStyle name="Purple" pivot="0" count="4" xr9:uid="{E5033B15-DEF9-4E53-9CD5-743BEEA85201}">
-      <tableStyleElement type="wholeTable" dxfId="63"/>
-      <tableStyleElement type="headerRow" dxfId="62"/>
-      <tableStyleElement type="firstRowStripe" dxfId="61"/>
-      <tableStyleElement type="secondRowStripe" dxfId="60"/>
+      <tableStyleElement type="wholeTable" dxfId="78"/>
+      <tableStyleElement type="headerRow" dxfId="77"/>
+      <tableStyleElement type="firstRowStripe" dxfId="76"/>
+      <tableStyleElement type="secondRowStripe" dxfId="75"/>
     </tableStyle>
     <tableStyle name="Purple-Main Table" pivot="0" count="6" xr9:uid="{857EDE21-F536-4B55-B74C-54E9A6FFB1EF}">
-      <tableStyleElement type="wholeTable" dxfId="59"/>
-      <tableStyleElement type="headerRow" dxfId="58"/>
-      <tableStyleElement type="totalRow" dxfId="57"/>
-      <tableStyleElement type="firstColumn" dxfId="56"/>
-      <tableStyleElement type="lastColumn" dxfId="55"/>
-      <tableStyleElement type="firstRowStripe" dxfId="54"/>
+      <tableStyleElement type="wholeTable" dxfId="74"/>
+      <tableStyleElement type="headerRow" dxfId="73"/>
+      <tableStyleElement type="totalRow" dxfId="72"/>
+      <tableStyleElement type="firstColumn" dxfId="71"/>
+      <tableStyleElement type="lastColumn" dxfId="70"/>
+      <tableStyleElement type="firstRowStripe" dxfId="69"/>
     </tableStyle>
   </tableStyles>
   <colors>
@@ -1116,50 +1246,94 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7D4CE7AD-7D83-4388-BABD-9691B076BBBB}" name="Table1" displayName="Table1" ref="K3:N6" totalsRowShown="0" headerRowDxfId="53" dataDxfId="52">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7D4CE7AD-7D83-4388-BABD-9691B076BBBB}" name="Table1" displayName="Table1" ref="K3:N6" totalsRowShown="0" headerRowDxfId="68" dataDxfId="4">
   <autoFilter ref="K3:N6" xr:uid="{7D4CE7AD-7D83-4388-BABD-9691B076BBBB}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{85D21381-7EAC-42E5-B4DC-5629383B9434}" name="x1" dataDxfId="51"/>
-    <tableColumn id="2" xr3:uid="{B77C55E8-DEEE-41C8-9AD6-50A09C54C70F}" name="x2" dataDxfId="50"/>
-    <tableColumn id="3" xr3:uid="{84052B22-E2E9-48E5-9C56-49F600EC333B}" name="x3" dataDxfId="49"/>
-    <tableColumn id="4" xr3:uid="{B0159775-53A4-430F-8281-9344C52FC0B5}" name="Igualdade" dataDxfId="48"/>
+    <tableColumn id="1" xr3:uid="{85D21381-7EAC-42E5-B4DC-5629383B9434}" name="x1" dataDxfId="3"/>
+    <tableColumn id="2" xr3:uid="{B77C55E8-DEEE-41C8-9AD6-50A09C54C70F}" name="x2" dataDxfId="2"/>
+    <tableColumn id="3" xr3:uid="{84052B22-E2E9-48E5-9C56-49F600EC333B}" name="x3" dataDxfId="1"/>
+    <tableColumn id="4" xr3:uid="{B0159775-53A4-430F-8281-9344C52FC0B5}" name="Igualdade" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
+<file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{A841A707-70AB-49C9-8520-7450D09B1881}" name="Table9" displayName="Table9" ref="E3:H8" totalsRowShown="0" headerRowDxfId="30" dataDxfId="27">
+  <autoFilter ref="E3:H8" xr:uid="{A841A707-70AB-49C9-8520-7450D09B1881}"/>
+  <tableColumns count="4">
+    <tableColumn id="2" xr3:uid="{D6AF72BE-448A-490A-9772-7329DB116300}" name="Ordem 1" dataDxfId="26"/>
+    <tableColumn id="3" xr3:uid="{1F32AAFA-7E62-4F56-A188-40D0C9524323}" name="Ordem 2" dataDxfId="25"/>
+    <tableColumn id="4" xr3:uid="{0FB7ADC9-CEAE-4D4A-B8EA-A39245C45C07}" name="Ordem 3" dataDxfId="24"/>
+    <tableColumn id="5" xr3:uid="{E04658AC-77E9-4307-9CAB-B0F45AF5F387}" name="Ordem 4" dataDxfId="23"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium4" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{14D190D1-A81B-4FD6-B90A-302E67B34006}" name="Table2" displayName="Table2" ref="B3:H14" totalsRowShown="0" headerRowDxfId="47" dataDxfId="46">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{14D190D1-A81B-4FD6-B90A-302E67B34006}" name="Table2" displayName="Table2" ref="B3:H14" totalsRowShown="0" headerRowDxfId="67" dataDxfId="66">
   <autoFilter ref="B3:H14" xr:uid="{14D190D1-A81B-4FD6-B90A-302E67B34006}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{6B7014C5-B393-4551-99C5-D69E22BCA2A1}" name="N" dataDxfId="45"/>
-    <tableColumn id="2" xr3:uid="{9EB42B44-08CA-489C-8E13-53DCC06784FF}" name="x1" dataDxfId="44"/>
-    <tableColumn id="3" xr3:uid="{01A8D2CE-D212-48B7-96F5-64004DE52476}" name="x2" dataDxfId="43"/>
-    <tableColumn id="4" xr3:uid="{71DE8002-5B74-4070-94C3-4A5E7EDAB7AD}" name="x3" dataDxfId="42"/>
-    <tableColumn id="5" xr3:uid="{631810F8-CA4D-4700-8459-C841DAF954A5}" name="Δx1" dataDxfId="41">
+    <tableColumn id="1" xr3:uid="{6B7014C5-B393-4551-99C5-D69E22BCA2A1}" name="N" dataDxfId="65"/>
+    <tableColumn id="2" xr3:uid="{9EB42B44-08CA-489C-8E13-53DCC06784FF}" name="x1" dataDxfId="64"/>
+    <tableColumn id="3" xr3:uid="{01A8D2CE-D212-48B7-96F5-64004DE52476}" name="x2" dataDxfId="63"/>
+    <tableColumn id="4" xr3:uid="{71DE8002-5B74-4070-94C3-4A5E7EDAB7AD}" name="x3" dataDxfId="62"/>
+    <tableColumn id="5" xr3:uid="{631810F8-CA4D-4700-8459-C841DAF954A5}" name="Δx1" dataDxfId="13">
       <calculatedColumnFormula>(Table2[[#This Row],[x1]]-C3)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{E17A8AB6-C9B6-4107-8E2B-201E756E149E}" name="Δx2" dataDxfId="40"/>
-    <tableColumn id="7" xr3:uid="{085FA800-56B0-4FCD-BCC0-A8979227F9EC}" name="x32" dataDxfId="39"/>
+    <tableColumn id="6" xr3:uid="{E17A8AB6-C9B6-4107-8E2B-201E756E149E}" name="Δx2" dataDxfId="12"/>
+    <tableColumn id="7" xr3:uid="{085FA800-56B0-4FCD-BCC0-A8979227F9EC}" name="Δx3" dataDxfId="11"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{CA5DF43D-7174-4083-99C4-5F5AB812AAC1}" name="Table3" displayName="Table3" ref="B3:I24" headerRowDxfId="38" dataDxfId="37">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{E0197C5E-3241-47A8-8729-E2EB6C2604C3}" name="Table15" displayName="Table15" ref="K3:N6" totalsRowShown="0" headerRowDxfId="22" dataDxfId="18">
+  <autoFilter ref="K3:N6" xr:uid="{7D4CE7AD-7D83-4388-BABD-9691B076BBBB}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{9C0E8CE7-0B5C-408D-B644-5AFEC9CBB560}" name="x1" dataDxfId="17"/>
+    <tableColumn id="2" xr3:uid="{7C879C62-B2B9-4693-9401-306433D95803}" name="x2" dataDxfId="16"/>
+    <tableColumn id="3" xr3:uid="{413963D5-BEDC-4CCF-810C-B86FBA2FAA7C}" name="x3" dataDxfId="15"/>
+    <tableColumn id="4" xr3:uid="{AE4C67C5-EA6A-4431-8927-84CF41885AEE}" name="Igualdade" dataDxfId="14"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{B943A5BF-3B1D-465F-8D50-9385891E339B}" name="Table211" displayName="Table211" ref="B3:H14" totalsRowShown="0" headerRowDxfId="21" dataDxfId="20">
+  <autoFilter ref="B3:H14" xr:uid="{14D190D1-A81B-4FD6-B90A-302E67B34006}"/>
+  <tableColumns count="7">
+    <tableColumn id="1" xr3:uid="{8065DED9-8664-46D8-93DC-CC8732AD69D8}" name="N" dataDxfId="19"/>
+    <tableColumn id="2" xr3:uid="{9A519208-E815-43A4-85EC-27D935381BC9}" name="x1" dataDxfId="7"/>
+    <tableColumn id="3" xr3:uid="{A70F5730-ED03-42AB-B8FF-C9536E45C565}" name="x2" dataDxfId="6"/>
+    <tableColumn id="4" xr3:uid="{920C6AE6-EFE5-445D-B656-F26F542BD1A0}" name="x3" dataDxfId="5"/>
+    <tableColumn id="5" xr3:uid="{89F4B0E3-6291-4209-8757-1542D3FE9528}" name="Δx1" dataDxfId="10">
+      <calculatedColumnFormula>(Table211[[#This Row],[x1]]-C3)</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="6" xr3:uid="{0E6C0825-7C58-49BD-9253-9C806425E24A}" name="Δx2" dataDxfId="9"/>
+    <tableColumn id="7" xr3:uid="{4AAED7FF-BEAF-42F6-8515-7002F299897A}" name="x32" dataDxfId="8"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{CA5DF43D-7174-4083-99C4-5F5AB812AAC1}" name="Table3" displayName="Table3" ref="B3:I24" headerRowDxfId="61" dataDxfId="60">
   <autoFilter ref="B3:I24" xr:uid="{CA5DF43D-7174-4083-99C4-5F5AB812AAC1}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{37116874-AE50-4C3C-9DD6-AB2C896C2C7B}" name="N" totalsRowLabel="Total" dataDxfId="36" totalsRowDxfId="35"/>
-    <tableColumn id="2" xr3:uid="{B3ECE0DE-56B1-4432-B529-258320B9F4C4}" name="a" dataDxfId="34" totalsRowDxfId="33"/>
-    <tableColumn id="3" xr3:uid="{70DDD3F5-2E57-4156-8F5F-A33E85AAF080}" name="b" dataDxfId="32" totalsRowDxfId="31"/>
-    <tableColumn id="4" xr3:uid="{21BAE3A7-01E6-44BE-916F-A00EF0BD2349}" name="x" dataDxfId="30" totalsRowDxfId="29">
-      <calculatedColumnFormula>ROUND((C4+D4)/20,6)</calculatedColumnFormula>
+    <tableColumn id="1" xr3:uid="{37116874-AE50-4C3C-9DD6-AB2C896C2C7B}" name="N" totalsRowLabel="Total" dataDxfId="59" totalsRowDxfId="58"/>
+    <tableColumn id="2" xr3:uid="{B3ECE0DE-56B1-4432-B529-258320B9F4C4}" name="a" dataDxfId="29" totalsRowDxfId="57"/>
+    <tableColumn id="3" xr3:uid="{70DDD3F5-2E57-4156-8F5F-A33E85AAF080}" name="b" dataDxfId="56" totalsRowDxfId="55"/>
+    <tableColumn id="4" xr3:uid="{21BAE3A7-01E6-44BE-916F-A00EF0BD2349}" name="x" dataDxfId="28" totalsRowDxfId="54">
+      <calculatedColumnFormula>ROUND((C4+D4)/2,6)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{E0978248-1055-4757-9B17-C79F5714BA77}" name="f(a)" dataDxfId="28" totalsRowDxfId="27"/>
-    <tableColumn id="6" xr3:uid="{13B90B5D-CAEB-4EE1-B7BE-D226D1A9FA9A}" name="f(b)" dataDxfId="26" totalsRowDxfId="25"/>
-    <tableColumn id="7" xr3:uid="{EC934254-DE38-462C-98AF-9C156DD09D2B}" name="f(x)" dataDxfId="24" totalsRowDxfId="23"/>
-    <tableColumn id="8" xr3:uid="{A927BBC3-28EB-4B87-B992-9E88692635BD}" name="b - a" totalsRowFunction="count" dataDxfId="22" totalsRowDxfId="21">
+    <tableColumn id="5" xr3:uid="{E0978248-1055-4757-9B17-C79F5714BA77}" name="f(a)" dataDxfId="53" totalsRowDxfId="52"/>
+    <tableColumn id="6" xr3:uid="{13B90B5D-CAEB-4EE1-B7BE-D226D1A9FA9A}" name="f(b)" dataDxfId="51" totalsRowDxfId="50"/>
+    <tableColumn id="7" xr3:uid="{EC934254-DE38-462C-98AF-9C156DD09D2B}" name="f(x)" dataDxfId="49" totalsRowDxfId="48"/>
+    <tableColumn id="8" xr3:uid="{A927BBC3-28EB-4B87-B992-9E88692635BD}" name="b - a" totalsRowFunction="count" dataDxfId="47" totalsRowDxfId="46">
       <calculatedColumnFormula>ROUND((D4-C4),6)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1167,25 +1341,25 @@
 </table>
 </file>
 
-<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{15D74070-D367-4512-875F-715997A7A4CC}" name="Table5" displayName="Table5" ref="B3:D7" totalsRowShown="0" headerRowDxfId="20" dataDxfId="19">
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{15D74070-D367-4512-875F-715997A7A4CC}" name="Table5" displayName="Table5" ref="B3:D7" totalsRowShown="0" headerRowDxfId="45" dataDxfId="44">
   <autoFilter ref="B3:D7" xr:uid="{15D74070-D367-4512-875F-715997A7A4CC}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{F24D6B1D-EC31-4715-8B13-B1D873AF007C}" name="i" dataDxfId="18"/>
-    <tableColumn id="2" xr3:uid="{E1EE6635-82E5-471C-861A-A6EB1A9C519C}" name="xi" dataDxfId="17"/>
-    <tableColumn id="3" xr3:uid="{DB64293B-D272-40FB-97E9-6143DF02F86C}" name="f(xi)" dataDxfId="16"/>
+    <tableColumn id="1" xr3:uid="{F24D6B1D-EC31-4715-8B13-B1D873AF007C}" name="i" dataDxfId="43"/>
+    <tableColumn id="2" xr3:uid="{E1EE6635-82E5-471C-861A-A6EB1A9C519C}" name="xi" dataDxfId="42"/>
+    <tableColumn id="3" xr3:uid="{DB64293B-D272-40FB-97E9-6143DF02F86C}" name="f(xi)" dataDxfId="41"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
-<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{4AC61E6D-D77A-45DD-AA5F-5C3EB7EFCE8F}" name="Table6" displayName="Table6" ref="E3:G7" totalsRowShown="0">
   <autoFilter ref="E3:G7" xr:uid="{4AC61E6D-D77A-45DD-AA5F-5C3EB7EFCE8F}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{BF05EAD5-6B5B-4B38-AA21-F4501A675942}" name="Termos"/>
-    <tableColumn id="2" xr3:uid="{06BBBFAF-5366-48ED-ACD0-7D2C066ADAF1}" name="lj(x)" dataDxfId="15"/>
-    <tableColumn id="3" xr3:uid="{16F7780B-AC0C-4643-819C-4E08B2A30137}" name="lj(x)*y(i)" dataDxfId="14">
+    <tableColumn id="2" xr3:uid="{06BBBFAF-5366-48ED-ACD0-7D2C066ADAF1}" name="lj(x)" dataDxfId="40"/>
+    <tableColumn id="3" xr3:uid="{16F7780B-AC0C-4643-819C-4E08B2A30137}" name="lj(x)*y(i)" dataDxfId="39">
       <calculatedColumnFormula>F4*D4</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1193,39 +1367,26 @@
 </table>
 </file>
 
-<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{731E2C8E-5713-4EF6-8135-A0CA41F14E9E}" name="Table7" displayName="Table7" ref="H3:I6" totalsRowShown="0" headerRowDxfId="13">
+<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{731E2C8E-5713-4EF6-8135-A0CA41F14E9E}" name="Table7" displayName="Table7" ref="H3:I6" totalsRowShown="0" headerRowDxfId="38">
   <autoFilter ref="H3:I6" xr:uid="{731E2C8E-5713-4EF6-8135-A0CA41F14E9E}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{2894579B-EE5C-45D7-B12F-0AA330900515}" name="Info" dataDxfId="12"/>
-    <tableColumn id="2" xr3:uid="{F06EEE62-E8C9-40BD-91DC-7CF74A06AC9F}" name="Número" dataDxfId="11"/>
+    <tableColumn id="1" xr3:uid="{2894579B-EE5C-45D7-B12F-0AA330900515}" name="Info" dataDxfId="37"/>
+    <tableColumn id="2" xr3:uid="{F06EEE62-E8C9-40BD-91DC-7CF74A06AC9F}" name="Número" dataDxfId="36"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="1" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
-<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D4C56C2C-992F-4CFD-B117-79873408CFD2}" name="Table8" displayName="Table8" ref="B3:D8" totalsRowShown="0" headerRowDxfId="10" dataDxfId="9">
+<file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D4C56C2C-992F-4CFD-B117-79873408CFD2}" name="Table8" displayName="Table8" ref="B3:D8" totalsRowShown="0" headerRowDxfId="35" dataDxfId="34">
   <autoFilter ref="B3:D8" xr:uid="{D4C56C2C-992F-4CFD-B117-79873408CFD2}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{2551832C-AB1B-438A-8807-BB5225C981A4}" name="i" dataDxfId="8"/>
-    <tableColumn id="2" xr3:uid="{D0B73F8B-855C-45B3-97D4-DAE4BA936537}" name="xi" dataDxfId="7"/>
-    <tableColumn id="3" xr3:uid="{16FE15A7-C99E-4391-89D9-85E3980CC8C6}" name="yi" dataDxfId="6"/>
+    <tableColumn id="1" xr3:uid="{2551832C-AB1B-438A-8807-BB5225C981A4}" name="i" dataDxfId="33"/>
+    <tableColumn id="2" xr3:uid="{D0B73F8B-855C-45B3-97D4-DAE4BA936537}" name="xi" dataDxfId="32"/>
+    <tableColumn id="3" xr3:uid="{16FE15A7-C99E-4391-89D9-85E3980CC8C6}" name="yi" dataDxfId="31"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{A841A707-70AB-49C9-8520-7450D09B1881}" name="Table9" displayName="Table9" ref="E3:H8" totalsRowShown="0" headerRowDxfId="5" dataDxfId="4">
-  <autoFilter ref="E3:H8" xr:uid="{A841A707-70AB-49C9-8520-7450D09B1881}"/>
-  <tableColumns count="4">
-    <tableColumn id="2" xr3:uid="{D6AF72BE-448A-490A-9772-7329DB116300}" name="Ordem 1" dataDxfId="3"/>
-    <tableColumn id="3" xr3:uid="{1F32AAFA-7E62-4F56-A188-40D0C9524323}" name="Ordem 2" dataDxfId="2"/>
-    <tableColumn id="4" xr3:uid="{0FB7ADC9-CEAE-4D4A-B8EA-A39245C45C07}" name="Ordem 3" dataDxfId="1"/>
-    <tableColumn id="5" xr3:uid="{E04658AC-77E9-4307-9CAB-B0F45AF5F387}" name="Ordem 4" dataDxfId="0"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium4" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -1535,7 +1696,7 @@
     <row r="1" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A1" s="1"/>
       <c r="B1" s="42" t="s">
-        <v>0</v>
+        <v>44</v>
       </c>
       <c r="C1" s="40"/>
       <c r="D1" s="40"/>
@@ -1547,20 +1708,20 @@
     <row r="2" spans="1:14" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A2" s="1"/>
       <c r="B2" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="39" t="s">
         <v>1</v>
-      </c>
-      <c r="C2" s="39" t="s">
-        <v>2</v>
       </c>
       <c r="D2" s="40"/>
       <c r="E2" s="40"/>
       <c r="F2" s="39" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G2" s="40"/>
       <c r="H2" s="41"/>
       <c r="K2" s="36" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L2" s="37"/>
       <c r="M2" s="37"/>
@@ -1568,37 +1729,37 @@
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.35">
       <c r="B3" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="D3" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="E3" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="F3" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="G3" s="62" t="s">
         <v>9</v>
       </c>
-      <c r="G3" s="1" t="s">
-        <v>10</v>
-      </c>
       <c r="H3" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="K3" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="L3" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="M3" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="N3" s="10" t="s">
         <v>11</v>
-      </c>
-      <c r="K3" s="11" t="s">
-        <v>6</v>
-      </c>
-      <c r="L3" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="M3" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="N3" s="10" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.35">
@@ -1617,313 +1778,337 @@
       <c r="F4" s="4">
         <v>0</v>
       </c>
-      <c r="G4" s="1">
+      <c r="G4" s="62">
         <v>0</v>
       </c>
       <c r="H4" s="5">
         <v>0</v>
       </c>
-      <c r="K4" s="4"/>
-      <c r="L4" s="4"/>
-      <c r="M4" s="4"/>
-      <c r="N4" s="2"/>
+      <c r="K4" s="4">
+        <v>8</v>
+      </c>
+      <c r="L4" s="4">
+        <v>-4</v>
+      </c>
+      <c r="M4" s="4">
+        <v>-3</v>
+      </c>
+      <c r="N4" s="2">
+        <v>14</v>
+      </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.35">
       <c r="B5" s="4">
         <v>1</v>
       </c>
-      <c r="C5" s="4" t="e">
+      <c r="C5" s="4">
         <f>ROUND(($N$4-$L$4*D4-$M$4*E4)/$K$4,3)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D5" s="1" t="e">
+        <v>1.75</v>
+      </c>
+      <c r="D5" s="1">
         <f>ROUND(($N$5-$K$5*C4-$M$5*E4)/$L$5,3)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E5" s="1" t="e">
+        <v>0.2</v>
+      </c>
+      <c r="E5" s="1">
         <f>ROUND(($N$6-$K$6*C4-$L$6*D4)/$M$6,3)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F5" s="4" t="e">
-        <f>(Table2[[#This Row],[x1]]-C4)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G5" s="1" t="e">
-        <f>(Table2[[#This Row],[x2]]-D4)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H5" s="5" t="e">
-        <f>(Table2[[#This Row],[x3]]-E4)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="K5" s="4"/>
-      <c r="L5" s="4"/>
-      <c r="M5" s="4"/>
-      <c r="N5" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="F5" s="4">
+        <f>ROUND((Table2[[#This Row],[x1]]-C4),3)</f>
+        <v>1.75</v>
+      </c>
+      <c r="G5" s="62">
+        <f>ROUND((Table2[[#This Row],[x2]]-D4),3)</f>
+        <v>0.2</v>
+      </c>
+      <c r="H5" s="5">
+        <f>ROUND((Table2[[#This Row],[x3]]-E4),3)</f>
+        <v>1</v>
+      </c>
+      <c r="K5" s="4">
+        <v>2</v>
+      </c>
+      <c r="L5" s="4">
+        <v>-5</v>
+      </c>
+      <c r="M5" s="4">
+        <v>3</v>
+      </c>
+      <c r="N5" s="2">
+        <v>-1</v>
+      </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.35">
       <c r="B6" s="4">
         <v>2</v>
       </c>
-      <c r="C6" s="4" t="e">
+      <c r="C6" s="4">
         <f t="shared" ref="C6:C14" si="0">ROUND(($N$4-$L$4*D5-$M$4*E5)/$K$4,3)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D6" s="1" t="e">
+        <v>2.2250000000000001</v>
+      </c>
+      <c r="D6" s="1">
         <f t="shared" ref="D6:D14" si="1">ROUND(($N$5-$K$5*C5-$M$5*E5)/$L$5,3)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E6" s="1" t="e">
+        <v>1.5</v>
+      </c>
+      <c r="E6" s="1">
         <f t="shared" ref="E6:E14" si="2">ROUND(($N$6-$K$6*C5-$L$6*D5)/$M$6,3)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F6" s="4" t="e">
-        <f>(Table2[[#This Row],[x1]]-C5)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G6" s="1" t="e">
-        <f>(Table2[[#This Row],[x2]]-D5)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H6" s="5" t="e">
-        <f>(Table2[[#This Row],[x3]]-E5)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="K6" s="6"/>
-      <c r="L6" s="6"/>
-      <c r="M6" s="6"/>
-      <c r="N6" s="3"/>
+        <v>1.5609999999999999</v>
+      </c>
+      <c r="F6" s="4">
+        <f>ROUND((Table2[[#This Row],[x1]]-C5),3)</f>
+        <v>0.47499999999999998</v>
+      </c>
+      <c r="G6" s="62">
+        <f>ROUND((Table2[[#This Row],[x2]]-D5),3)</f>
+        <v>1.3</v>
+      </c>
+      <c r="H6" s="5">
+        <f>ROUND((Table2[[#This Row],[x3]]-E5),3)</f>
+        <v>0.56100000000000005</v>
+      </c>
+      <c r="K6" s="6">
+        <v>-3</v>
+      </c>
+      <c r="L6" s="6">
+        <v>1</v>
+      </c>
+      <c r="M6" s="6">
+        <v>9</v>
+      </c>
+      <c r="N6" s="3">
+        <v>9</v>
+      </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.35">
       <c r="B7" s="4">
         <v>3</v>
       </c>
-      <c r="C7" s="4" t="e">
+      <c r="C7" s="4">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D7" s="1" t="e">
+        <v>3.085</v>
+      </c>
+      <c r="D7" s="1">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E7" s="1" t="e">
+        <v>2.0270000000000001</v>
+      </c>
+      <c r="E7" s="1">
         <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F7" s="4" t="e">
-        <f>(Table2[[#This Row],[x1]]-C6)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G7" s="1" t="e">
-        <f>(Table2[[#This Row],[x2]]-D6)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H7" s="5" t="e">
-        <f>(Table2[[#This Row],[x3]]-E6)</f>
-        <v>#DIV/0!</v>
+        <v>1.575</v>
+      </c>
+      <c r="F7" s="4">
+        <f>ROUND((Table2[[#This Row],[x1]]-C6),3)</f>
+        <v>0.86</v>
+      </c>
+      <c r="G7" s="62">
+        <f>ROUND((Table2[[#This Row],[x2]]-D6),3)</f>
+        <v>0.52700000000000002</v>
+      </c>
+      <c r="H7" s="5">
+        <f>ROUND((Table2[[#This Row],[x3]]-E6),3)</f>
+        <v>1.4E-2</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.35">
       <c r="B8" s="4">
         <v>4</v>
       </c>
-      <c r="C8" s="4" t="e">
+      <c r="C8" s="4">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D8" s="1" t="e">
+        <v>3.3540000000000001</v>
+      </c>
+      <c r="D8" s="1">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E8" s="1" t="e">
+        <v>2.379</v>
+      </c>
+      <c r="E8" s="1">
         <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F8" s="4" t="e">
-        <f>(Table2[[#This Row],[x1]]-C7)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G8" s="1" t="e">
-        <f>(Table2[[#This Row],[x2]]-D7)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H8" s="5" t="e">
-        <f>(Table2[[#This Row],[x3]]-E7)</f>
-        <v>#DIV/0!</v>
+        <v>1.8029999999999999</v>
+      </c>
+      <c r="F8" s="4">
+        <f>ROUND((Table2[[#This Row],[x1]]-C7),3)</f>
+        <v>0.26900000000000002</v>
+      </c>
+      <c r="G8" s="62">
+        <f>ROUND((Table2[[#This Row],[x2]]-D7),3)</f>
+        <v>0.35199999999999998</v>
+      </c>
+      <c r="H8" s="5">
+        <f>ROUND((Table2[[#This Row],[x3]]-E7),3)</f>
+        <v>0.22800000000000001</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.35">
       <c r="B9" s="4">
         <v>5</v>
       </c>
-      <c r="C9" s="4" t="e">
+      <c r="C9" s="4">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D9" s="1" t="e">
+        <v>3.6160000000000001</v>
+      </c>
+      <c r="D9" s="1">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E9" s="1" t="e">
+        <v>2.6230000000000002</v>
+      </c>
+      <c r="E9" s="1">
         <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F9" s="4" t="e">
-        <f>(Table2[[#This Row],[x1]]-C8)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G9" s="1" t="e">
-        <f>(Table2[[#This Row],[x2]]-D8)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H9" s="5" t="e">
-        <f>(Table2[[#This Row],[x3]]-E8)</f>
-        <v>#DIV/0!</v>
+        <v>1.8540000000000001</v>
+      </c>
+      <c r="F9" s="4">
+        <f>ROUND((Table2[[#This Row],[x1]]-C8),3)</f>
+        <v>0.26200000000000001</v>
+      </c>
+      <c r="G9" s="62">
+        <f>ROUND((Table2[[#This Row],[x2]]-D8),3)</f>
+        <v>0.24399999999999999</v>
+      </c>
+      <c r="H9" s="5">
+        <f>ROUND((Table2[[#This Row],[x3]]-E8),3)</f>
+        <v>5.0999999999999997E-2</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.35">
       <c r="B10" s="4">
         <v>6</v>
       </c>
-      <c r="C10" s="4" t="e">
+      <c r="C10" s="4">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D10" s="1" t="e">
+        <v>3.7570000000000001</v>
+      </c>
+      <c r="D10" s="1">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E10" s="1" t="e">
+        <v>2.7589999999999999</v>
+      </c>
+      <c r="E10" s="1">
         <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F10" s="4" t="e">
-        <f>(Table2[[#This Row],[x1]]-C9)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G10" s="1" t="e">
-        <f>(Table2[[#This Row],[x2]]-D9)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H10" s="5" t="e">
-        <f>(Table2[[#This Row],[x3]]-E9)</f>
-        <v>#DIV/0!</v>
+        <v>1.9139999999999999</v>
+      </c>
+      <c r="F10" s="4">
+        <f>ROUND((Table2[[#This Row],[x1]]-C9),3)</f>
+        <v>0.14099999999999999</v>
+      </c>
+      <c r="G10" s="62">
+        <f>ROUND((Table2[[#This Row],[x2]]-D9),3)</f>
+        <v>0.13600000000000001</v>
+      </c>
+      <c r="H10" s="5">
+        <f>ROUND((Table2[[#This Row],[x3]]-E9),3)</f>
+        <v>0.06</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.35">
       <c r="B11" s="4">
         <v>7</v>
       </c>
-      <c r="C11" s="4" t="e">
+      <c r="C11" s="4">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D11" s="1" t="e">
+        <v>3.847</v>
+      </c>
+      <c r="D11" s="1">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E11" s="1" t="e">
+        <v>2.851</v>
+      </c>
+      <c r="E11" s="1">
         <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F11" s="4" t="e">
-        <f>(Table2[[#This Row],[x1]]-C10)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G11" s="1" t="e">
-        <f>(Table2[[#This Row],[x2]]-D10)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H11" s="5" t="e">
-        <f>(Table2[[#This Row],[x3]]-E10)</f>
-        <v>#DIV/0!</v>
+        <v>1.946</v>
+      </c>
+      <c r="F11" s="4">
+        <f>ROUND((Table2[[#This Row],[x1]]-C10),3)</f>
+        <v>0.09</v>
+      </c>
+      <c r="G11" s="62">
+        <f>ROUND((Table2[[#This Row],[x2]]-D10),3)</f>
+        <v>9.1999999999999998E-2</v>
+      </c>
+      <c r="H11" s="5">
+        <f>ROUND((Table2[[#This Row],[x3]]-E10),3)</f>
+        <v>3.2000000000000001E-2</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.35">
       <c r="B12" s="4">
         <v>8</v>
       </c>
-      <c r="C12" s="4" t="e">
+      <c r="C12" s="4">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D12" s="1" t="e">
+        <v>3.9049999999999998</v>
+      </c>
+      <c r="D12" s="1">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E12" s="1" t="e">
+        <v>2.9060000000000001</v>
+      </c>
+      <c r="E12" s="1">
         <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F12" s="4" t="e">
-        <f>(Table2[[#This Row],[x1]]-C11)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G12" s="1" t="e">
-        <f>(Table2[[#This Row],[x2]]-D11)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H12" s="5" t="e">
-        <f>(Table2[[#This Row],[x3]]-E11)</f>
-        <v>#DIV/0!</v>
+        <v>1.966</v>
+      </c>
+      <c r="F12" s="4">
+        <f>ROUND((Table2[[#This Row],[x1]]-C11),3)</f>
+        <v>5.8000000000000003E-2</v>
+      </c>
+      <c r="G12" s="62">
+        <f>ROUND((Table2[[#This Row],[x2]]-D11),3)</f>
+        <v>5.5E-2</v>
+      </c>
+      <c r="H12" s="5">
+        <f>ROUND((Table2[[#This Row],[x3]]-E11),3)</f>
+        <v>0.02</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.35">
       <c r="B13" s="4">
         <v>9</v>
       </c>
-      <c r="C13" s="4" t="e">
+      <c r="C13" s="4">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D13" s="1" t="e">
+        <v>3.94</v>
+      </c>
+      <c r="D13" s="1">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E13" s="1" t="e">
+        <v>2.9420000000000002</v>
+      </c>
+      <c r="E13" s="1">
         <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F13" s="4" t="e">
-        <f>(Table2[[#This Row],[x1]]-C12)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G13" s="1" t="e">
-        <f>(Table2[[#This Row],[x2]]-D12)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H13" s="5" t="e">
-        <f>(Table2[[#This Row],[x3]]-E12)</f>
-        <v>#DIV/0!</v>
+        <v>1.9790000000000001</v>
+      </c>
+      <c r="F13" s="4">
+        <f>ROUND((Table2[[#This Row],[x1]]-C12),3)</f>
+        <v>3.5000000000000003E-2</v>
+      </c>
+      <c r="G13" s="62">
+        <f>ROUND((Table2[[#This Row],[x2]]-D12),3)</f>
+        <v>3.5999999999999997E-2</v>
+      </c>
+      <c r="H13" s="5">
+        <f>ROUND((Table2[[#This Row],[x3]]-E12),3)</f>
+        <v>1.2999999999999999E-2</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.35">
       <c r="B14" s="6">
         <v>10</v>
       </c>
-      <c r="C14" s="6" t="e">
+      <c r="C14" s="6">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D14" s="7" t="e">
+        <v>3.9630000000000001</v>
+      </c>
+      <c r="D14" s="7">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E14" s="7" t="e">
+        <v>2.9630000000000001</v>
+      </c>
+      <c r="E14" s="7">
         <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F14" s="6" t="e">
-        <f>(Table2[[#This Row],[x1]]-C13)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G14" s="7" t="e">
-        <f>(Table2[[#This Row],[x2]]-D13)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H14" s="8" t="e">
-        <f>(Table2[[#This Row],[x3]]-E13)</f>
-        <v>#DIV/0!</v>
+        <v>1.986</v>
+      </c>
+      <c r="F14" s="6">
+        <f>ROUND((Table2[[#This Row],[x1]]-C13),3)</f>
+        <v>2.3E-2</v>
+      </c>
+      <c r="G14" s="7">
+        <f>ROUND((Table2[[#This Row],[x2]]-D13),3)</f>
+        <v>2.1000000000000001E-2</v>
+      </c>
+      <c r="H14" s="8">
+        <f>ROUND((Table2[[#This Row],[x3]]-E13),3)</f>
+        <v>7.0000000000000001E-3</v>
       </c>
     </row>
   </sheetData>
@@ -1942,13 +2127,459 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B39DD5BD-E6FA-4B21-A745-88D78DF2F2C6}">
+  <dimension ref="A1:N15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="14" max="14" width="12.1796875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A1" s="1"/>
+      <c r="B1" s="42" t="s">
+        <v>45</v>
+      </c>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
+      <c r="G1" s="40"/>
+      <c r="H1" s="41"/>
+    </row>
+    <row r="2" spans="1:14" ht="18.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A2" s="1"/>
+      <c r="B2" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="39" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" s="40"/>
+      <c r="E2" s="41"/>
+      <c r="F2" s="39" t="s">
+        <v>2</v>
+      </c>
+      <c r="G2" s="40"/>
+      <c r="H2" s="41"/>
+      <c r="K2" s="36" t="s">
+        <v>3</v>
+      </c>
+      <c r="L2" s="37"/>
+      <c r="M2" s="37"/>
+      <c r="N2" s="38"/>
+    </row>
+    <row r="3" spans="1:14" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="B3" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D3" s="62" t="s">
+        <v>6</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="G3" s="62" t="s">
+        <v>9</v>
+      </c>
+      <c r="H3" s="61" t="s">
+        <v>10</v>
+      </c>
+      <c r="K3" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="L3" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="M3" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="N3" s="10" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="B4" s="4">
+        <v>0</v>
+      </c>
+      <c r="C4" s="4">
+        <v>0</v>
+      </c>
+      <c r="D4" s="62">
+        <v>0</v>
+      </c>
+      <c r="E4" s="5">
+        <v>0</v>
+      </c>
+      <c r="F4" s="4">
+        <v>0</v>
+      </c>
+      <c r="G4" s="62">
+        <v>0</v>
+      </c>
+      <c r="H4" s="5">
+        <v>0</v>
+      </c>
+      <c r="K4" s="4">
+        <v>8</v>
+      </c>
+      <c r="L4" s="4">
+        <v>-4</v>
+      </c>
+      <c r="M4" s="4">
+        <v>-3</v>
+      </c>
+      <c r="N4" s="2">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="B5" s="4">
+        <v>1</v>
+      </c>
+      <c r="C5" s="4">
+        <f>ROUND((($N$4-L4*D4-M4*E4)/$K$4),3)</f>
+        <v>1.75</v>
+      </c>
+      <c r="D5" s="62">
+        <f>ROUND((($N$5-$K$5*C5-$M$5*E4)/$L$5),3)</f>
+        <v>0.9</v>
+      </c>
+      <c r="E5" s="5">
+        <f>ROUND((($N$6-$K$6*C5-$L$6*D5)/$M$6),3)</f>
+        <v>1.4830000000000001</v>
+      </c>
+      <c r="F5" s="4">
+        <f>ROUND((Table211[[#This Row],[x1]]-C4),3)</f>
+        <v>1.75</v>
+      </c>
+      <c r="G5" s="62">
+        <f>ROUND((Table211[[#This Row],[x2]]-D4),3)</f>
+        <v>0.9</v>
+      </c>
+      <c r="H5" s="5">
+        <f>ROUND((Table211[[#This Row],[x3]]-E4),3)</f>
+        <v>1.4830000000000001</v>
+      </c>
+      <c r="K5" s="4">
+        <v>2</v>
+      </c>
+      <c r="L5" s="4">
+        <v>-5</v>
+      </c>
+      <c r="M5" s="4">
+        <v>3</v>
+      </c>
+      <c r="N5" s="2">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="B6" s="4">
+        <v>2</v>
+      </c>
+      <c r="C6" s="4">
+        <f>ROUND((($N$4-L5*D5-M5*E5)/$K$4),3)</f>
+        <v>1.756</v>
+      </c>
+      <c r="D6" s="62">
+        <f>ROUND((($N$5-$K$5*C6-$M$5*E5)/$L$5),3)</f>
+        <v>1.792</v>
+      </c>
+      <c r="E6" s="5">
+        <f>ROUND((($N$6-$K$6*C6-$L$6*D6)/$M$6),3)</f>
+        <v>1.3859999999999999</v>
+      </c>
+      <c r="F6" s="4">
+        <f>ROUND((Table211[[#This Row],[x1]]-C5),3)</f>
+        <v>6.0000000000000001E-3</v>
+      </c>
+      <c r="G6" s="62">
+        <f>ROUND((Table211[[#This Row],[x2]]-D5),3)</f>
+        <v>0.89200000000000002</v>
+      </c>
+      <c r="H6" s="5">
+        <f>ROUND((Table211[[#This Row],[x3]]-E5),3)</f>
+        <v>-9.7000000000000003E-2</v>
+      </c>
+      <c r="K6" s="6">
+        <v>-3</v>
+      </c>
+      <c r="L6" s="6">
+        <v>1</v>
+      </c>
+      <c r="M6" s="6">
+        <v>9</v>
+      </c>
+      <c r="N6" s="3">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="B7" s="4">
+        <v>3</v>
+      </c>
+      <c r="C7" s="4">
+        <f>ROUND((($N$4-L6*D6-M6*E6)/$K$4),3)</f>
+        <v>-3.3000000000000002E-2</v>
+      </c>
+      <c r="D7" s="62">
+        <f>ROUND((($N$5-$K$5*C7-$M$5*E6)/$L$5),3)</f>
+        <v>1.018</v>
+      </c>
+      <c r="E7" s="5">
+        <f>ROUND((($N$6-$K$6*C7-$L$6*D7)/$M$6),3)</f>
+        <v>0.876</v>
+      </c>
+      <c r="F7" s="4">
+        <f>ROUND((Table211[[#This Row],[x1]]-C6),3)</f>
+        <v>-1.7889999999999999</v>
+      </c>
+      <c r="G7" s="62">
+        <f>ROUND((Table211[[#This Row],[x2]]-D6),3)</f>
+        <v>-0.77400000000000002</v>
+      </c>
+      <c r="H7" s="5">
+        <f>ROUND((Table211[[#This Row],[x3]]-E6),3)</f>
+        <v>-0.51</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="B8" s="4">
+        <v>4</v>
+      </c>
+      <c r="C8" s="4">
+        <f>ROUND((($N$4-L7*D7-M7*E7)/$K$4),3)</f>
+        <v>1.75</v>
+      </c>
+      <c r="D8" s="62">
+        <f>ROUND((($N$5-$K$5*C8-$M$5*E7)/$L$5),3)</f>
+        <v>1.4259999999999999</v>
+      </c>
+      <c r="E8" s="5">
+        <f>ROUND((($N$6-$K$6*C8-$L$6*D8)/$M$6),3)</f>
+        <v>1.425</v>
+      </c>
+      <c r="F8" s="4">
+        <f>ROUND((Table211[[#This Row],[x1]]-C7),3)</f>
+        <v>1.7829999999999999</v>
+      </c>
+      <c r="G8" s="62">
+        <f>ROUND((Table211[[#This Row],[x2]]-D7),3)</f>
+        <v>0.40799999999999997</v>
+      </c>
+      <c r="H8" s="5">
+        <f>ROUND((Table211[[#This Row],[x3]]-E7),3)</f>
+        <v>0.54900000000000004</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="B9" s="4">
+        <v>5</v>
+      </c>
+      <c r="C9" s="4">
+        <f>ROUND((($N$4-L8*D8-M8*E8)/$K$4),3)</f>
+        <v>1.75</v>
+      </c>
+      <c r="D9" s="62">
+        <f>ROUND((($N$5-$K$5*C9-$M$5*E8)/$L$5),3)</f>
+        <v>1.7549999999999999</v>
+      </c>
+      <c r="E9" s="5">
+        <f>ROUND((($N$6-$K$6*C9-$L$6*D9)/$M$6),3)</f>
+        <v>1.3879999999999999</v>
+      </c>
+      <c r="F9" s="4">
+        <f>ROUND((Table211[[#This Row],[x1]]-C8),3)</f>
+        <v>0</v>
+      </c>
+      <c r="G9" s="62">
+        <f>ROUND((Table211[[#This Row],[x2]]-D8),3)</f>
+        <v>0.32900000000000001</v>
+      </c>
+      <c r="H9" s="5">
+        <f>ROUND((Table211[[#This Row],[x3]]-E8),3)</f>
+        <v>-3.6999999999999998E-2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="B10" s="4">
+        <v>6</v>
+      </c>
+      <c r="C10" s="4">
+        <f>ROUND((($N$4-L9*D9-M9*E9)/$K$4),3)</f>
+        <v>1.75</v>
+      </c>
+      <c r="D10" s="62">
+        <f>ROUND((($N$5-$K$5*C10-$M$5*E9)/$L$5),3)</f>
+        <v>1.7330000000000001</v>
+      </c>
+      <c r="E10" s="5">
+        <f>ROUND((($N$6-$K$6*C10-$L$6*D10)/$M$6),3)</f>
+        <v>1.391</v>
+      </c>
+      <c r="F10" s="4">
+        <f>ROUND((Table211[[#This Row],[x1]]-C9),3)</f>
+        <v>0</v>
+      </c>
+      <c r="G10" s="62">
+        <f>ROUND((Table211[[#This Row],[x2]]-D9),3)</f>
+        <v>-2.1999999999999999E-2</v>
+      </c>
+      <c r="H10" s="5">
+        <f>ROUND((Table211[[#This Row],[x3]]-E9),3)</f>
+        <v>3.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="B11" s="4">
+        <v>7</v>
+      </c>
+      <c r="C11" s="4">
+        <f>ROUND((($N$4-L10*D10-M10*E10)/$K$4),3)</f>
+        <v>1.75</v>
+      </c>
+      <c r="D11" s="62">
+        <f>ROUND((($N$5-$K$5*C11-$M$5*E10)/$L$5),3)</f>
+        <v>1.7350000000000001</v>
+      </c>
+      <c r="E11" s="5">
+        <f>ROUND((($N$6-$K$6*C11-$L$6*D11)/$M$6),3)</f>
+        <v>1.391</v>
+      </c>
+      <c r="F11" s="4">
+        <f>ROUND((Table211[[#This Row],[x1]]-C10),3)</f>
+        <v>0</v>
+      </c>
+      <c r="G11" s="62">
+        <f>ROUND((Table211[[#This Row],[x2]]-D10),3)</f>
+        <v>2E-3</v>
+      </c>
+      <c r="H11" s="5">
+        <f>ROUND((Table211[[#This Row],[x3]]-E10),3)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="B12" s="4">
+        <v>8</v>
+      </c>
+      <c r="C12" s="4">
+        <f>ROUND((($N$4-L11*D11-M11*E11)/$K$4),3)</f>
+        <v>1.75</v>
+      </c>
+      <c r="D12" s="62">
+        <f>ROUND((($N$5-$K$5*C12-$M$5*E11)/$L$5),3)</f>
+        <v>1.7350000000000001</v>
+      </c>
+      <c r="E12" s="5">
+        <f>ROUND((($N$6-$K$6*C12-$L$6*D12)/$M$6),3)</f>
+        <v>1.391</v>
+      </c>
+      <c r="F12" s="4">
+        <f>ROUND((Table211[[#This Row],[x1]]-C11),3)</f>
+        <v>0</v>
+      </c>
+      <c r="G12" s="62">
+        <f>ROUND((Table211[[#This Row],[x2]]-D11),3)</f>
+        <v>0</v>
+      </c>
+      <c r="H12" s="5">
+        <f>ROUND((Table211[[#This Row],[x3]]-E11),3)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="B13" s="4">
+        <v>9</v>
+      </c>
+      <c r="C13" s="4">
+        <f>ROUND((($N$4-L12*D12-M12*E12)/$K$4),3)</f>
+        <v>1.75</v>
+      </c>
+      <c r="D13" s="62">
+        <f>ROUND((($N$5-$K$5*C13-$M$5*E12)/$L$5),3)</f>
+        <v>1.7350000000000001</v>
+      </c>
+      <c r="E13" s="5">
+        <f>ROUND((($N$6-$K$6*C13-$L$6*D13)/$M$6),3)</f>
+        <v>1.391</v>
+      </c>
+      <c r="F13" s="4">
+        <f>ROUND((Table211[[#This Row],[x1]]-C12),3)</f>
+        <v>0</v>
+      </c>
+      <c r="G13" s="62">
+        <f>ROUND((Table211[[#This Row],[x2]]-D12),3)</f>
+        <v>0</v>
+      </c>
+      <c r="H13" s="5">
+        <f>ROUND((Table211[[#This Row],[x3]]-E12),3)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="B14" s="6">
+        <v>10</v>
+      </c>
+      <c r="C14" s="6">
+        <f>ROUND((($N$4-L13*D13-M13*E13)/$K$4),3)</f>
+        <v>1.75</v>
+      </c>
+      <c r="D14" s="7">
+        <f>ROUND((($N$5-$K$5*C14-$M$5*E13)/$L$5),3)</f>
+        <v>1.7350000000000001</v>
+      </c>
+      <c r="E14" s="8">
+        <f>ROUND((($N$6-$K$6*C14-$L$6*D14)/$M$6),3)</f>
+        <v>1.391</v>
+      </c>
+      <c r="F14" s="6">
+        <f>ROUND((Table211[[#This Row],[x1]]-C13),3)</f>
+        <v>0</v>
+      </c>
+      <c r="G14" s="7">
+        <f>ROUND((Table211[[#This Row],[x2]]-D13),3)</f>
+        <v>0</v>
+      </c>
+      <c r="H14" s="8">
+        <f>ROUND((Table211[[#This Row],[x3]]-E13),3)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="F15" s="63"/>
+      <c r="G15" s="63"/>
+      <c r="H15" s="63"/>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="B1:H1"/>
+    <mergeCell ref="C2:E2"/>
+    <mergeCell ref="F2:H2"/>
+    <mergeCell ref="K2:N2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="2">
+    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4BF5D226-2B48-4C24-A633-83AF724169BB}">
   <dimension ref="B1:I24"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B1" s="43" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C1" s="44"/>
       <c r="D1" s="44"/>
@@ -1960,7 +2591,7 @@
     </row>
     <row r="2" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B2" s="43" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C2" s="44"/>
       <c r="D2" s="44"/>
@@ -1972,45 +2603,45 @@
     </row>
     <row r="3" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B3" s="15" t="s">
-        <v>5</v>
-      </c>
-      <c r="C3" s="15" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="D3" s="15" t="s">
+      <c r="E3" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="E3" s="15" t="s">
+      <c r="F3" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="F3" s="15" t="s">
+      <c r="G3" s="16" t="s">
         <v>18</v>
       </c>
-      <c r="G3" s="16" t="s">
+      <c r="H3" s="16" t="s">
         <v>19</v>
       </c>
-      <c r="H3" s="16" t="s">
+      <c r="I3" s="14" t="s">
         <v>20</v>
-      </c>
-      <c r="I3" s="14" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="4" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B4" s="4">
         <v>0</v>
       </c>
-      <c r="C4" s="4"/>
+      <c r="C4" s="2"/>
       <c r="D4" s="4"/>
       <c r="E4" s="4">
-        <f t="shared" ref="E4:E24" si="0">ROUND((C4+D4)/20,6)</f>
+        <f>ROUND((C4+D4)/2,6)</f>
         <v>0</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="1"/>
       <c r="H4" s="1"/>
       <c r="I4" s="2">
-        <f t="shared" ref="I4:I24" si="1">ROUND((D4-C4),6)</f>
+        <f t="shared" ref="I4:I24" si="0">ROUND((D4-C4),6)</f>
         <v>0</v>
       </c>
     </row>
@@ -2018,8 +2649,8 @@
       <c r="B5" s="4">
         <v>1</v>
       </c>
-      <c r="C5" s="4">
-        <f>ROUND(IF(F4-H4&lt;0,C4,E4),6)</f>
+      <c r="C5" s="2">
+        <f>ROUND(IF(F4*H4&lt;0,C4,E4),6)</f>
         <v>0</v>
       </c>
       <c r="D5" s="4">
@@ -2027,14 +2658,14 @@
         <v>0</v>
       </c>
       <c r="E5" s="4">
-        <f t="shared" si="0"/>
+        <f>ROUND((C5+D5)/2,6)</f>
         <v>0</v>
       </c>
       <c r="F5" s="4"/>
       <c r="G5" s="1"/>
       <c r="H5" s="1"/>
       <c r="I5" s="2">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
@@ -2042,23 +2673,23 @@
       <c r="B6" s="4">
         <v>2</v>
       </c>
-      <c r="C6" s="4">
-        <f t="shared" ref="C6:C24" si="2">ROUND(IF(F5-H5&lt;0,C5,E5),6)</f>
+      <c r="C6" s="2">
+        <f>ROUND(IF(F5*H5&lt;0,C5,E5),6)</f>
         <v>0</v>
       </c>
       <c r="D6" s="4">
-        <f t="shared" ref="D6:D24" si="3">ROUND(IF(G5*H5&lt;0,D5,E5),6)</f>
+        <f t="shared" ref="D6:D24" si="1">ROUND(IF(G5*H5&lt;0,D5,E5),6)</f>
         <v>0</v>
       </c>
       <c r="E6" s="4">
-        <f t="shared" si="0"/>
+        <f>ROUND((C6+D6)/2,6)</f>
         <v>0</v>
       </c>
       <c r="F6" s="4"/>
       <c r="G6" s="1"/>
       <c r="H6" s="1"/>
       <c r="I6" s="2">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
@@ -2066,23 +2697,23 @@
       <c r="B7" s="4">
         <v>3</v>
       </c>
-      <c r="C7" s="4">
-        <f t="shared" si="2"/>
+      <c r="C7" s="2">
+        <f>ROUND(IF(F6*H6&lt;0,C6,E6),6)</f>
         <v>0</v>
       </c>
       <c r="D7" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="E7" s="4">
-        <f t="shared" si="0"/>
+        <f>ROUND((C7+D7)/2,6)</f>
         <v>0</v>
       </c>
       <c r="F7" s="4"/>
       <c r="G7" s="1"/>
       <c r="H7" s="1"/>
       <c r="I7" s="2">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
@@ -2090,23 +2721,23 @@
       <c r="B8" s="4">
         <v>4</v>
       </c>
-      <c r="C8" s="4">
-        <f t="shared" si="2"/>
+      <c r="C8" s="2">
+        <f>ROUND(IF(F7*H7&lt;0,C7,E7),6)</f>
         <v>0</v>
       </c>
       <c r="D8" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="E8" s="4">
-        <f t="shared" si="0"/>
+        <f>ROUND((C8+D8)/2,6)</f>
         <v>0</v>
       </c>
       <c r="F8" s="4"/>
       <c r="G8" s="1"/>
       <c r="H8" s="1"/>
       <c r="I8" s="2">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
@@ -2114,23 +2745,23 @@
       <c r="B9" s="4">
         <v>5</v>
       </c>
-      <c r="C9" s="4">
-        <f t="shared" si="2"/>
+      <c r="C9" s="2">
+        <f>ROUND(IF(F8*H8&lt;0,C8,E8),6)</f>
         <v>0</v>
       </c>
       <c r="D9" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="E9" s="4">
-        <f t="shared" si="0"/>
+        <f>ROUND((C9+D9)/2,6)</f>
         <v>0</v>
       </c>
       <c r="F9" s="4"/>
       <c r="G9" s="1"/>
       <c r="H9" s="1"/>
       <c r="I9" s="2">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
@@ -2138,23 +2769,23 @@
       <c r="B10" s="4">
         <v>6</v>
       </c>
-      <c r="C10" s="4">
-        <f t="shared" si="2"/>
+      <c r="C10" s="2">
+        <f>ROUND(IF(F9*H9&lt;0,C9,E9),6)</f>
         <v>0</v>
       </c>
       <c r="D10" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="E10" s="4">
-        <f t="shared" si="0"/>
+        <f>ROUND((C10+D10)/2,6)</f>
         <v>0</v>
       </c>
       <c r="F10" s="4"/>
       <c r="G10" s="1"/>
       <c r="H10" s="1"/>
       <c r="I10" s="2">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
@@ -2162,23 +2793,23 @@
       <c r="B11" s="4">
         <v>7</v>
       </c>
-      <c r="C11" s="4">
-        <f t="shared" si="2"/>
+      <c r="C11" s="2">
+        <f>ROUND(IF(F10*H10&lt;0,C10,E10),6)</f>
         <v>0</v>
       </c>
       <c r="D11" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="E11" s="4">
-        <f t="shared" si="0"/>
+        <f>ROUND((C11+D11)/2,6)</f>
         <v>0</v>
       </c>
       <c r="F11" s="4"/>
       <c r="G11" s="1"/>
       <c r="H11" s="1"/>
       <c r="I11" s="2">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
@@ -2186,23 +2817,23 @@
       <c r="B12" s="4">
         <v>8</v>
       </c>
-      <c r="C12" s="4">
-        <f t="shared" si="2"/>
+      <c r="C12" s="2">
+        <f>ROUND(IF(F11*H11&lt;0,C11,E11),6)</f>
         <v>0</v>
       </c>
       <c r="D12" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="E12" s="4">
-        <f t="shared" si="0"/>
+        <f>ROUND((C12+D12)/2,6)</f>
         <v>0</v>
       </c>
       <c r="F12" s="4"/>
       <c r="G12" s="1"/>
       <c r="H12" s="1"/>
       <c r="I12" s="2">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
@@ -2210,23 +2841,23 @@
       <c r="B13" s="4">
         <v>9</v>
       </c>
-      <c r="C13" s="4">
-        <f t="shared" si="2"/>
+      <c r="C13" s="2">
+        <f>ROUND(IF(F12*H12&lt;0,C12,E12),6)</f>
         <v>0</v>
       </c>
       <c r="D13" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="E13" s="4">
-        <f t="shared" si="0"/>
+        <f>ROUND((C13+D13)/2,6)</f>
         <v>0</v>
       </c>
       <c r="F13" s="4"/>
       <c r="G13" s="1"/>
       <c r="H13" s="1"/>
       <c r="I13" s="2">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
@@ -2234,23 +2865,23 @@
       <c r="B14" s="4">
         <v>10</v>
       </c>
-      <c r="C14" s="4">
-        <f t="shared" si="2"/>
+      <c r="C14" s="2">
+        <f>ROUND(IF(F13*H13&lt;0,C13,E13),6)</f>
         <v>0</v>
       </c>
       <c r="D14" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="E14" s="4">
-        <f t="shared" si="0"/>
+        <f>ROUND((C14+D14)/2,6)</f>
         <v>0</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="1"/>
       <c r="H14" s="1"/>
       <c r="I14" s="2">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
@@ -2258,23 +2889,23 @@
       <c r="B15" s="4">
         <v>11</v>
       </c>
-      <c r="C15" s="4">
-        <f t="shared" si="2"/>
+      <c r="C15" s="2">
+        <f>ROUND(IF(F14*H14&lt;0,C14,E14),6)</f>
         <v>0</v>
       </c>
       <c r="D15" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="E15" s="4">
-        <f t="shared" si="0"/>
+        <f>ROUND((C15+D15)/2,6)</f>
         <v>0</v>
       </c>
       <c r="F15" s="4"/>
       <c r="G15" s="1"/>
       <c r="H15" s="1"/>
       <c r="I15" s="2">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
@@ -2282,23 +2913,23 @@
       <c r="B16" s="4">
         <v>12</v>
       </c>
-      <c r="C16" s="4">
-        <f t="shared" si="2"/>
+      <c r="C16" s="2">
+        <f>ROUND(IF(F15*H15&lt;0,C15,E15),6)</f>
         <v>0</v>
       </c>
       <c r="D16" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="E16" s="4">
-        <f t="shared" si="0"/>
+        <f>ROUND((C16+D16)/2,6)</f>
         <v>0</v>
       </c>
       <c r="F16" s="4"/>
       <c r="G16" s="1"/>
       <c r="H16" s="1"/>
       <c r="I16" s="2">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
@@ -2306,23 +2937,23 @@
       <c r="B17" s="4">
         <v>13</v>
       </c>
-      <c r="C17" s="4">
-        <f t="shared" si="2"/>
+      <c r="C17" s="2">
+        <f>ROUND(IF(F16*H16&lt;0,C16,E16),6)</f>
         <v>0</v>
       </c>
       <c r="D17" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="E17" s="4">
-        <f t="shared" si="0"/>
+        <f>ROUND((C17+D17)/2,6)</f>
         <v>0</v>
       </c>
       <c r="F17" s="4"/>
       <c r="G17" s="1"/>
       <c r="H17" s="1"/>
       <c r="I17" s="2">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
@@ -2330,23 +2961,23 @@
       <c r="B18" s="4">
         <v>14</v>
       </c>
-      <c r="C18" s="4">
-        <f t="shared" si="2"/>
+      <c r="C18" s="2">
+        <f>ROUND(IF(F17*H17&lt;0,C17,E17),6)</f>
         <v>0</v>
       </c>
       <c r="D18" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="E18" s="4">
-        <f t="shared" si="0"/>
+        <f>ROUND((C18+D18)/2,6)</f>
         <v>0</v>
       </c>
       <c r="F18" s="4"/>
       <c r="G18" s="1"/>
       <c r="H18" s="1"/>
       <c r="I18" s="2">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
@@ -2354,23 +2985,23 @@
       <c r="B19" s="4">
         <v>15</v>
       </c>
-      <c r="C19" s="4">
-        <f t="shared" si="2"/>
+      <c r="C19" s="2">
+        <f>ROUND(IF(F18*H18&lt;0,C18,E18),6)</f>
         <v>0</v>
       </c>
       <c r="D19" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="E19" s="4">
-        <f t="shared" si="0"/>
+        <f>ROUND((C19+D19)/2,6)</f>
         <v>0</v>
       </c>
       <c r="F19" s="4"/>
       <c r="G19" s="1"/>
       <c r="H19" s="1"/>
       <c r="I19" s="2">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
@@ -2378,23 +3009,23 @@
       <c r="B20" s="4">
         <v>16</v>
       </c>
-      <c r="C20" s="4">
-        <f t="shared" si="2"/>
+      <c r="C20" s="2">
+        <f>ROUND(IF(F19*H19&lt;0,C19,E19),6)</f>
         <v>0</v>
       </c>
       <c r="D20" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="E20" s="4">
-        <f t="shared" si="0"/>
+        <f>ROUND((C20+D20)/2,6)</f>
         <v>0</v>
       </c>
       <c r="F20" s="4"/>
       <c r="G20" s="1"/>
       <c r="H20" s="1"/>
       <c r="I20" s="2">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
@@ -2402,23 +3033,23 @@
       <c r="B21" s="4">
         <v>17</v>
       </c>
-      <c r="C21" s="4">
-        <f t="shared" si="2"/>
+      <c r="C21" s="2">
+        <f>ROUND(IF(F20*H20&lt;0,C20,E20),6)</f>
         <v>0</v>
       </c>
       <c r="D21" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="E21" s="4">
-        <f t="shared" si="0"/>
+        <f>ROUND((C21+D21)/2,6)</f>
         <v>0</v>
       </c>
       <c r="F21" s="4"/>
       <c r="G21" s="1"/>
       <c r="H21" s="1"/>
       <c r="I21" s="2">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
@@ -2426,23 +3057,23 @@
       <c r="B22" s="4">
         <v>18</v>
       </c>
-      <c r="C22" s="4">
-        <f t="shared" si="2"/>
+      <c r="C22" s="2">
+        <f>ROUND(IF(F21*H21&lt;0,C21,E21),6)</f>
         <v>0</v>
       </c>
       <c r="D22" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="E22" s="4">
-        <f t="shared" si="0"/>
+        <f>ROUND((C22+D22)/2,6)</f>
         <v>0</v>
       </c>
       <c r="F22" s="4"/>
       <c r="G22" s="1"/>
       <c r="H22" s="1"/>
       <c r="I22" s="2">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
@@ -2450,23 +3081,23 @@
       <c r="B23" s="4">
         <v>19</v>
       </c>
-      <c r="C23" s="4">
-        <f t="shared" si="2"/>
+      <c r="C23" s="2">
+        <f>ROUND(IF(F22*H22&lt;0,C22,E22),6)</f>
         <v>0</v>
       </c>
       <c r="D23" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="E23" s="4">
-        <f t="shared" si="0"/>
+        <f>ROUND((C23+D23)/2,6)</f>
         <v>0</v>
       </c>
       <c r="F23" s="4"/>
       <c r="G23" s="1"/>
       <c r="H23" s="1"/>
       <c r="I23" s="2">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
@@ -2474,23 +3105,23 @@
       <c r="B24" s="6">
         <v>20</v>
       </c>
-      <c r="C24" s="6">
-        <f t="shared" si="2"/>
+      <c r="C24" s="3">
+        <f>ROUND(IF(F23*H23&lt;0,C23,E23),6)</f>
         <v>0</v>
       </c>
       <c r="D24" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="E24" s="6">
-        <f t="shared" si="0"/>
+        <f>ROUND((C24+D24)/2,6)</f>
         <v>0</v>
       </c>
       <c r="F24" s="6"/>
       <c r="G24" s="7"/>
       <c r="H24" s="7"/>
       <c r="I24" s="3">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
@@ -2507,7 +3138,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{10562F7C-477D-47B7-A744-5FA395DF9716}">
   <dimension ref="B1:Q20"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -2520,7 +3151,7 @@
   <sheetData>
     <row r="1" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B1" s="53" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C1" s="54"/>
       <c r="D1" s="54"/>
@@ -2536,17 +3167,17 @@
     </row>
     <row r="2" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B2" s="47" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C2" s="48"/>
       <c r="D2" s="48"/>
       <c r="E2" s="51" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F2" s="52"/>
       <c r="G2" s="52"/>
       <c r="H2" s="49" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="I2" s="50"/>
       <c r="N2" s="18"/>
@@ -2556,28 +3187,28 @@
     </row>
     <row r="3" spans="2:17" ht="18.5" x14ac:dyDescent="0.45">
       <c r="B3" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="D3" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="E3" s="22" t="s">
         <v>28</v>
       </c>
-      <c r="E3" s="22" t="s">
+      <c r="F3" t="s">
         <v>29</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" s="20" t="s">
         <v>30</v>
       </c>
-      <c r="G3" s="20" t="s">
+      <c r="H3" s="27" t="s">
         <v>31</v>
       </c>
-      <c r="H3" s="27" t="s">
+      <c r="I3" s="23" t="s">
         <v>32</v>
-      </c>
-      <c r="I3" s="23" t="s">
-        <v>33</v>
       </c>
       <c r="J3" s="17"/>
       <c r="K3" s="17"/>
@@ -2604,7 +3235,7 @@
         <v>#DIV/0!</v>
       </c>
       <c r="H4" s="28" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="I4" s="24"/>
       <c r="J4" s="19"/>
@@ -2632,7 +3263,7 @@
         <v>#DIV/0!</v>
       </c>
       <c r="H5" s="28" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I5" s="24"/>
       <c r="J5" s="19"/>
@@ -2660,7 +3291,7 @@
         <v>#DIV/0!</v>
       </c>
       <c r="H6" s="28" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="I6" s="24" t="e">
         <f>(G4+G5+G6+G7)</f>
@@ -2691,7 +3322,7 @@
         <v>#DIV/0!</v>
       </c>
       <c r="H7" s="42" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="I7" s="46"/>
       <c r="J7" s="19"/>
@@ -2872,7 +3503,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B14FEB47-A731-4433-A198-E50957206D09}">
   <dimension ref="B1:H8"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -2886,7 +3517,7 @@
   <sheetData>
     <row r="1" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B1" s="56" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C1" s="57"/>
       <c r="D1" s="57"/>
@@ -2897,12 +3528,12 @@
     </row>
     <row r="2" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B2" s="56" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C2" s="57"/>
       <c r="D2" s="58"/>
       <c r="E2" s="59" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F2" s="59"/>
       <c r="G2" s="59"/>
@@ -2910,25 +3541,25 @@
     </row>
     <row r="3" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B3" s="31" t="s">
+        <v>25</v>
+      </c>
+      <c r="C3" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="C3" s="13" t="s">
-        <v>27</v>
-      </c>
       <c r="D3" s="32" t="s">
+        <v>39</v>
+      </c>
+      <c r="E3" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="E3" s="13" t="s">
+      <c r="F3" s="13" t="s">
         <v>41</v>
       </c>
-      <c r="F3" s="13" t="s">
+      <c r="G3" s="13" t="s">
         <v>42</v>
       </c>
-      <c r="G3" s="13" t="s">
+      <c r="H3" s="32" t="s">
         <v>43</v>
-      </c>
-      <c r="H3" s="32" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="4" spans="2:8" x14ac:dyDescent="0.35">
@@ -2961,7 +3592,7 @@
       <c r="C5" s="1"/>
       <c r="D5" s="5"/>
       <c r="E5" s="19" t="e">
-        <f t="shared" ref="E5:E7" si="0">(D6-D5)/(C6-C5)</f>
+        <f>(D6-D5)/(C6-C5)</f>
         <v>#DIV/0!</v>
       </c>
       <c r="F5" s="19" t="e">
@@ -2984,7 +3615,7 @@
       <c r="C6" s="1"/>
       <c r="D6" s="5"/>
       <c r="E6" s="19" t="e">
-        <f t="shared" si="0"/>
+        <f>(D7-D6)/(C7-C6)</f>
         <v>#DIV/0!</v>
       </c>
       <c r="F6" s="19" t="e">
@@ -3007,7 +3638,7 @@
       <c r="C7" s="1"/>
       <c r="D7" s="5"/>
       <c r="E7" s="19" t="e">
-        <f t="shared" si="0"/>
+        <f>(D8-D7)/(C8-C7)</f>
         <v>#DIV/0!</v>
       </c>
       <c r="F7" s="30" t="e">

</xml_diff>